<commit_message>
Update project requests management table
</commit_message>
<xml_diff>
--- a/PJ依頼事項管理表.xlsx
+++ b/PJ依頼事項管理表.xlsx
@@ -5,27 +5,38 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\umesk\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ProjectManagement\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2650ED8-1BFD-43F0-8A54-47A0D883FDEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D381407-A8D8-4BB9-9A9A-F735F264A985}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5280" yWindow="5280" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2660" yWindow="2660" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="台帳" sheetId="1" r:id="rId1"/>
     <sheet name="回答一覧" sheetId="2" r:id="rId2"/>
     <sheet name="team定義" sheetId="3" r:id="rId3"/>
+    <sheet name="PJ情報" sheetId="5" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="67">
-  <si>
-    <t>依頼事項一覧</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="50">
   <si>
     <t>依頼内容</t>
   </si>
@@ -48,9 +59,6 @@
     <t>#2</t>
   </si>
   <si>
-    <t>～～～について、YYYをお願いします</t>
-  </si>
-  <si>
     <t>#3</t>
   </si>
   <si>
@@ -114,115 +122,163 @@
     <t>チームNo</t>
   </si>
   <si>
+    <t>team_1</t>
+  </si>
+  <si>
+    <t>xxxです。</t>
+  </si>
+  <si>
+    <t>team_2</t>
+  </si>
+  <si>
+    <t>team_3</t>
+  </si>
+  <si>
+    <t>team_4</t>
+  </si>
+  <si>
+    <t>team_5</t>
+  </si>
+  <si>
+    <t>担当者_2</t>
+  </si>
+  <si>
+    <t>担当者_3</t>
+  </si>
+  <si>
+    <t>担当者_4</t>
+  </si>
+  <si>
+    <t>担当者_5</t>
+  </si>
+  <si>
+    <t>依頼中</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>依頼ID</t>
+    <rPh sb="0" eb="2">
+      <t>イライ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>team_3</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
     <t>回答内容</t>
-  </si>
-  <si>
-    <t>team_1</t>
-  </si>
-  <si>
-    <t>xxxです。</t>
-  </si>
-  <si>
-    <t>team_2</t>
-  </si>
-  <si>
-    <t>team_3</t>
-  </si>
-  <si>
-    <t>team_4</t>
-  </si>
-  <si>
-    <t>team_5</t>
-  </si>
-  <si>
-    <t>担当者_1</t>
-  </si>
-  <si>
-    <t>担当者_2</t>
-  </si>
-  <si>
-    <t>担当者_3</t>
-  </si>
-  <si>
-    <t>担当者_4</t>
-  </si>
-  <si>
-    <t>担当者_5</t>
-  </si>
-  <si>
-    <t>xxx1_1@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx1_2@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx1_3@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx1_4@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx1_5@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx2_1@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx2_2@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx2_3@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx2_4@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx2_5@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx3_1@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx3_2@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx3_3@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx3_4@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx3_5@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx4_1@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx4_2@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx4_3@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx4_4@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx4_5@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx5_1@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx5_2@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx5_3@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx5_4@gmail.com</t>
-  </si>
-  <si>
-    <t>xxx5_5@gmail.com</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>担当者</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>_1</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>Project XYZ</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>PM_メールアドレス</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>#2</t>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>～～～について、</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>YYY</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>をお願いします</t>
+    </r>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <t>リマインド送付時cc_</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>メールアドレス</t>
+    </r>
+    <rPh sb="5" eb="8">
+      <t>ソウフジ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <r>
+      <t>Project</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="ＭＳ ゴシック"/>
+        <family val="3"/>
+        <charset val="128"/>
+      </rPr>
+      <t>名</t>
+    </r>
+    <rPh sb="7" eb="8">
+      <t>メイ</t>
+    </rPh>
+    <phoneticPr fontId="2"/>
+  </si>
+  <si>
+    <t>xxx@outlook.jp</t>
+    <phoneticPr fontId="2"/>
   </si>
 </sst>
 </file>
@@ -232,7 +288,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="m/d"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -251,6 +307,50 @@
       <family val="3"/>
       <charset val="128"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="ＭＳ ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="ＭＳ ゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="3">
@@ -291,16 +391,26 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="176" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="ハイパーリンク" xfId="1" builtinId="8"/>
     <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -314,10 +424,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -535,64 +641,64 @@
       <c r="E2" s="1"/>
     </row>
     <row r="3" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>2</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>3</v>
       </c>
     </row>
     <row r="4" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" s="2" t="s">
         <v>4</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>5</v>
       </c>
       <c r="D4" s="3">
         <v>46166</v>
       </c>
-      <c r="E4" s="2" t="s">
-        <v>6</v>
+      <c r="E4" s="4" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>8</v>
+      <c r="B5" s="6" t="s">
+        <v>45</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>46</v>
       </c>
       <c r="D5" s="3">
         <v>46167</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D6" s="3">
         <v>46168</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="7" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -600,7 +706,7 @@
     </row>
     <row r="8" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2"/>
@@ -608,7 +714,7 @@
     </row>
     <row r="9" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2"/>
@@ -616,7 +722,7 @@
     </row>
     <row r="10" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
@@ -624,7 +730,7 @@
     </row>
     <row r="11" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -632,7 +738,7 @@
     </row>
     <row r="12" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2"/>
@@ -640,7 +746,7 @@
     </row>
     <row r="13" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B13" s="2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
@@ -648,7 +754,7 @@
     </row>
     <row r="14" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B14" s="2" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
@@ -656,7 +762,7 @@
     </row>
     <row r="15" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B15" s="2" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
@@ -664,7 +770,7 @@
     </row>
     <row r="16" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B16" s="2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
@@ -672,7 +778,7 @@
     </row>
     <row r="17" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B17" s="2" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
@@ -680,7 +786,7 @@
     </row>
     <row r="18" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B18" s="2" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -688,7 +794,7 @@
     </row>
     <row r="19" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B19" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
@@ -696,7 +802,7 @@
     </row>
     <row r="20" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B20" s="2" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -704,7 +810,7 @@
     </row>
     <row r="21" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B21" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -712,7 +818,7 @@
     </row>
     <row r="22" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B22" s="2" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -720,7 +826,7 @@
     </row>
     <row r="23" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B23" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -745,160 +851,160 @@
   <sheetData>
     <row r="2" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C2" s="1"/>
       <c r="D2" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>30</v>
+        <v>27</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C3" s="2" t="str">
         <f>VLOOKUP(B3,台帳!B:C,2,FALSE)</f>
         <v>～～～について、XXXをお願いします</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C4" s="2" t="str">
         <f>VLOOKUP(B4,台帳!B:C,2,FALSE)</f>
         <v>～～～について、XXXをお願いします</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C5" s="2" t="str">
         <f>VLOOKUP(B5,台帳!B:C,2,FALSE)</f>
         <v>～～～について、XXXをお願いします</v>
       </c>
-      <c r="D5" s="2" t="s">
-        <v>34</v>
+      <c r="D5" s="6" t="s">
+        <v>40</v>
       </c>
       <c r="E5" s="2"/>
     </row>
     <row r="6" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C6" s="2" t="str">
         <f>VLOOKUP(B6,台帳!B:C,2,FALSE)</f>
         <v>～～～について、XXXをお願いします</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="E6" s="2"/>
     </row>
     <row r="7" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C7" s="2" t="str">
         <f>VLOOKUP(B7,台帳!B:C,2,FALSE)</f>
         <v>～～～について、XXXをお願いします</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="8" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B8" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C8" s="2" t="str">
         <f>VLOOKUP(B8,台帳!B:C,2,FALSE)</f>
         <v>～～～について、YYYをお願いします</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B9" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C9" s="2" t="str">
         <f>VLOOKUP(B9,台帳!B:C,2,FALSE)</f>
         <v>～～～について、YYYをお願いします</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="10" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B10" s="2" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="C10" s="2" t="str">
         <f>VLOOKUP(B10,台帳!B:C,2,FALSE)</f>
         <v>～～～について、YYYをお願いします</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="11" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B11" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C11" s="2" t="str">
         <f>VLOOKUP(B11,台帳!B:C,2,FALSE)</f>
         <v>～～～について、ZZZをお願いします</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="12" spans="2:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B12" s="2" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C12" s="2" t="str">
         <f>VLOOKUP(B12,台帳!B:C,2,FALSE)</f>
         <v>～～～について、ZZZをお願いします</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -916,129 +1022,171 @@
   <dimension ref="B2:G7"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="7" width="17.36328125" customWidth="1"/>
+    <col min="3" max="7" width="26.54296875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="1"/>
-      <c r="C2" s="1" t="s">
+      <c r="B2" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C2" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>37</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="3" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>42</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="F3" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G3" s="2" t="s">
-        <v>46</v>
+        <v>28</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G3" s="9" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>48</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F4" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="G4" s="2" t="s">
-        <v>51</v>
+        <v>30</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F4" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G4" s="9" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B5" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>52</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>53</v>
-      </c>
-      <c r="E5" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="F5" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="G5" s="2" t="s">
-        <v>56</v>
+        <v>31</v>
+      </c>
+      <c r="C5" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D5" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E5" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F5" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G5" s="9" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B6" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F6" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="G6" s="2" t="s">
-        <v>61</v>
+        <v>32</v>
+      </c>
+      <c r="C6" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D6" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G6" s="9" t="s">
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="2:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B7" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>62</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="G7" s="2" t="s">
-        <v>66</v>
+        <v>33</v>
+      </c>
+      <c r="C7" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="D7" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="E7" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>49</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DB56C08C-CD36-40FF-80EE-90F796267627}">
+  <dimension ref="B2:C4"/>
+  <sheetFormatPr defaultRowHeight="12.5" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="18.36328125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.81640625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B2" s="10" t="s">
+        <v>48</v>
+      </c>
+      <c r="C2" s="10" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B3" s="10" t="s">
+        <v>44</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.25">
+      <c r="B4" s="10" t="s">
+        <v>47</v>
+      </c>
+      <c r="C4" s="9" t="s">
+        <v>49</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>